<commit_message>
feat(upload): expand basic tree XLSForm
</commit_message>
<xml_diff>
--- a/apps/bumicerts/public/templates/tree-data-basic-xlsform.xlsx
+++ b/apps/bumicerts/public/templates/tree-data-basic-xlsform.xlsx
@@ -56,7 +56,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -246,6 +246,150 @@
         </is>
       </c>
       <c r="H5"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>height</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Tree Height (m)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Tree height in meters.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>. &gt; 0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Height must be greater than 0.</t>
+        </is>
+      </c>
+      <c r="H6"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>dbh</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DBH (cm)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Diameter at breast height in centimeters.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>. &gt; 0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>DBH must be greater than 0.</t>
+        </is>
+      </c>
+      <c r="H7"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>decimal</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>diameter</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Diameter (cm)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Basal, stem, crown, or other measured diameter in centimeters.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>. &gt; 0</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Diameter must be greater than 0.</t>
+        </is>
+      </c>
+      <c r="H8"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>photo_tree</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Whole Tree Photo</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Take or choose a whole-tree photo. Export Kobo Media Attachments ZIP with your CSV.</t>
+        </is>
+      </c>
+      <c r="F9"/>
+      <c r="G9"/>
+      <c r="H9"/>
     </row>
   </sheetData>
 </worksheet>
@@ -322,7 +466,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>

</xml_diff>